<commit_message>
added ortools script and constraints file
</commit_message>
<xml_diff>
--- a/addresses/mock_google_data/distance_coords_cache.xlsx
+++ b/addresses/mock_google_data/distance_coords_cache.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D64"/>
+  <dimension ref="A1:D76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -747,14 +747,14 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>אבני נזר 21, מודיעין עילית</t>
+          <t>אבני נזר 12, מודיעין עילית</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>31.9346348</v>
+        <v>31.934894</v>
       </c>
       <c r="C19" t="n">
-        <v>35.0430467</v>
+        <v>35.043743</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -783,14 +783,14 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>הריטבא 8, מודיעין עילית</t>
+          <t>משך חכמה 60, מודיעין עילית</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>31.9273875</v>
+        <v>31.9337067</v>
       </c>
       <c r="C21" t="n">
-        <v>35.04697220000001</v>
+        <v>35.0397399</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -801,14 +801,14 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>חזון איש 10, מודיעין עילית</t>
+          <t>נתיבות המשפט 3, מודיעין עילית</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>31.9222529</v>
+        <v>31.9336533</v>
       </c>
       <c r="C22" t="n">
-        <v>35.0504504</v>
+        <v>35.04736200000001</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -819,14 +819,14 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>חזון דוד 17, מודיעין עילית</t>
+          <t>רבי יהודה הנשיא 20, מודיעין עילית</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>31.9257054</v>
+        <v>31.9385733</v>
       </c>
       <c r="C23" t="n">
-        <v>35.0404598</v>
+        <v>35.0430685</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -837,14 +837,14 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>חזון דוד 27, מודיעין עילית</t>
+          <t>רבי יהודה הנשיא 26, מודיעין עילית</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>31.9243742</v>
+        <v>31.938572</v>
       </c>
       <c r="C24" t="n">
-        <v>35.0435251</v>
+        <v>35.0454471</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -855,14 +855,14 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>מסילת יוסף 19, מודיעין עילית</t>
+          <t>רבי עקיבא 14, מודיעין עילית</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>31.926859</v>
+        <v>31.94064719999999</v>
       </c>
       <c r="C25" t="n">
-        <v>35.0426428</v>
+        <v>35.04146740000001</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -873,14 +873,14 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>משך חכמה 60, מודיעין עילית</t>
+          <t>רשבי 3, מודיעין עילית</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>31.9337067</v>
+        <v>31.9377883</v>
       </c>
       <c r="C26" t="n">
-        <v>35.0397399</v>
+        <v>35.0386719</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -891,14 +891,14 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>נתיבות המשפט 71, מודיעין עילית</t>
+          <t>רשבי 12, מודיעין עילית</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>31.9259043</v>
+        <v>31.9374409</v>
       </c>
       <c r="C27" t="n">
-        <v>35.0444855</v>
+        <v>35.0406868</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -909,14 +909,14 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>נתיבות המשפט 85, מודיעין עילית</t>
+          <t>רשבי 22, מודיעין עילית</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>31.9245194</v>
+        <v>31.9370797</v>
       </c>
       <c r="C28" t="n">
-        <v>35.0419395</v>
+        <v>35.0430294</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -927,14 +927,14 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>נתיבות המשפט 93, מודיעין עילית</t>
+          <t>רשבי 32, מודיעין עילית</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>31.9257393</v>
+        <v>31.9369865</v>
       </c>
       <c r="C29" t="n">
-        <v>35.0407657</v>
+        <v>35.0450276</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -945,14 +945,14 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>נתיבות שלום 11, מודיעין עילית</t>
+          <t>שדי חמד 15, מודיעין עילית</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>31.92844</v>
+        <v>31.93349499999999</v>
       </c>
       <c r="C30" t="n">
-        <v>35.0504422</v>
+        <v>35.042305</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -963,14 +963,14 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>קצות החושן 8, מודיעין עילית</t>
+          <t>אשר לשלמה 1, מודיעין עילית</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>31.9279674</v>
+        <v>31.9232333</v>
       </c>
       <c r="C31" t="n">
-        <v>35.0420405</v>
+        <v>35.0458679</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -981,14 +981,14 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>רבי יהודה הנשיא 21, מודיעין עילית</t>
+          <t>הריטבא 8, מודיעין עילית</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>31.9395316</v>
+        <v>31.9273875</v>
       </c>
       <c r="C32" t="n">
-        <v>35.042133</v>
+        <v>35.04697220000001</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -999,14 +999,14 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>רבי יהודה הנשיא 26, מודיעין עילית</t>
+          <t>חזון איש 7, מודיעין עילית</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>31.938572</v>
+        <v>31.9226253</v>
       </c>
       <c r="C33" t="n">
-        <v>35.0454471</v>
+        <v>35.049516</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -1017,14 +1017,14 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>רבי עקיבא 14, מודיעין עילית</t>
+          <t>חזון איש 15, מודיעין עילית</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>31.94064719999999</v>
+        <v>31.9221798</v>
       </c>
       <c r="C34" t="n">
-        <v>35.04146740000001</v>
+        <v>35.0516505</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -1035,14 +1035,14 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>רמבם 18, מודיעין עילית</t>
+          <t>חזון איש 23, מודיעין עילית</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>31.9293284</v>
+        <v>31.92194</v>
       </c>
       <c r="C35" t="n">
-        <v>35.0465972</v>
+        <v>35.0532167</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -1053,14 +1053,14 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>רשבי 3, מודיעין עילית</t>
+          <t>חזון איש 26, מודיעין עילית</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>31.9377883</v>
+        <v>31.9222529</v>
       </c>
       <c r="C36" t="n">
-        <v>35.0386719</v>
+        <v>35.0504504</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
@@ -1071,14 +1071,14 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>רשבי 12, מודיעין עילית</t>
+          <t>חזון דוד 17, מודיעין עילית</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>31.9374409</v>
+        <v>31.9257054</v>
       </c>
       <c r="C37" t="n">
-        <v>35.0406868</v>
+        <v>35.0404598</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -1089,14 +1089,14 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>רשבי 37, מודיעין עילית</t>
+          <t>חזון דוד 25, מודיעין עילית</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>31.9373403</v>
+        <v>31.924268</v>
       </c>
       <c r="C38" t="n">
-        <v>35.044505</v>
+        <v>35.043069</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -1107,14 +1107,14 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>שאגת אריה 1, מודיעין עילית</t>
+          <t>חפץ חיים 21, מודיעין עילית</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>31.9290753</v>
+        <v>31.9301503</v>
       </c>
       <c r="C39" t="n">
-        <v>35.04182249999999</v>
+        <v>35.042627</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -1125,14 +1125,14 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>שדי חמד 28, מודיעין עילית</t>
+          <t>מסילת יוסף 14, מודיעין עילית</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>31.9328825</v>
+        <v>31.9312516</v>
       </c>
       <c r="C40" t="n">
-        <v>35.0410932</v>
+        <v>35.045036</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -1143,14 +1143,14 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>שערי תשובה 6, מודיעין עילית</t>
+          <t>מסילת יוסף 19, מודיעין עילית</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>31.927077</v>
+        <v>31.926859</v>
       </c>
       <c r="C41" t="n">
-        <v>35.03831</v>
+        <v>35.0426428</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -1161,14 +1161,14 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>אשל 5, רכסים</t>
+          <t>מרומי שדה 3, מודיעין עילית</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>32.7537724</v>
+        <v>31.9286714</v>
       </c>
       <c r="C42" t="n">
-        <v>35.107609</v>
+        <v>35.0440405</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
@@ -1179,14 +1179,14 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>דקל 2, רכסים</t>
+          <t>נתיבות המשפט 59, מודיעין עילית</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>32.7531176</v>
+        <v>31.9278568</v>
       </c>
       <c r="C43" t="n">
-        <v>35.10734310000001</v>
+        <v>35.0452741</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
@@ -1197,14 +1197,14 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>הדס 4, רכסים</t>
+          <t>נתיבות המשפט 71, מודיעין עילית</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>32.7551946</v>
+        <v>31.9259043</v>
       </c>
       <c r="C44" t="n">
-        <v>35.1066628</v>
+        <v>35.0444855</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -1215,14 +1215,14 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>הדקל 30, רכסים</t>
+          <t>נתיבות המשפט 85, מודיעין עילית</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>32.7552473</v>
+        <v>31.9245194</v>
       </c>
       <c r="C45" t="n">
-        <v>35.1072159</v>
+        <v>35.0419395</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
@@ -1233,14 +1233,14 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>הורדים 4, רכסים</t>
+          <t>נתיבות המשפט 93, מודיעין עילית</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>32.755216</v>
+        <v>31.9257393</v>
       </c>
       <c r="C46" t="n">
-        <v>35.0965091</v>
+        <v>35.0407657</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -1251,14 +1251,14 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>הכלניות 1, רכסים</t>
+          <t>נתיבות המשפט 107, מודיעין עילית</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>32.7541406</v>
+        <v>31.927568</v>
       </c>
       <c r="C47" t="n">
-        <v>35.0975422</v>
+        <v>35.038982</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -1269,14 +1269,14 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>הכלניות 32, רכסים</t>
+          <t>נתיבות שלום 11, מודיעין עילית</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>32.753939</v>
+        <v>31.92844</v>
       </c>
       <c r="C48" t="n">
-        <v>35.09969299999999</v>
+        <v>35.0504422</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -1287,14 +1287,14 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>הכלניות 47, רכסים</t>
+          <t>קצות החושן 8, מודיעין עילית</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>32.7535253</v>
+        <v>31.9279674</v>
       </c>
       <c r="C49" t="n">
-        <v>35.10205910000001</v>
+        <v>35.0420405</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
@@ -1305,14 +1305,14 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>הנרקיסים 24, רכסים</t>
+          <t>קצות החושן 17, מודיעין עילית</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>32.7564592</v>
+        <v>31.9283181</v>
       </c>
       <c r="C50" t="n">
-        <v>35.0993751</v>
+        <v>35.0395641</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -1323,14 +1323,14 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>הרב קוק 12, רכסים</t>
+          <t>רמבם 18, מודיעין עילית</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>32.7465011</v>
+        <v>31.9293284</v>
       </c>
       <c r="C51" t="n">
-        <v>35.1002575</v>
+        <v>35.0465972</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
@@ -1341,14 +1341,14 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>הרב קוק 26, רכסים</t>
+          <t>שאגת אריה 1, מודיעין עילית</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>32.7472521</v>
+        <v>31.9290753</v>
       </c>
       <c r="C52" t="n">
-        <v>35.1022188</v>
+        <v>35.04182249999999</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
@@ -1359,14 +1359,14 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>הרימונים 16, רכסים</t>
+          <t>שערי תשובה 6, מודיעין עילית</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>32.7499409</v>
+        <v>31.927077</v>
       </c>
       <c r="C53" t="n">
-        <v>35.0985743</v>
+        <v>35.03831</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
@@ -1377,14 +1377,14 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>השקד 13, רכסים</t>
+          <t>אשל 5, רכסים</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>32.752189</v>
+        <v>32.7537724</v>
       </c>
       <c r="C54" t="n">
-        <v>35.103784</v>
+        <v>35.107609</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
@@ -1395,14 +1395,14 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>השקד 14, רכסים</t>
+          <t>דקל 2, רכסים</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>32.750799</v>
+        <v>32.7531176</v>
       </c>
       <c r="C55" t="n">
-        <v>35.102316</v>
+        <v>35.10734310000001</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
@@ -1413,14 +1413,14 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>השקד 40, רכסים</t>
+          <t>הדס 4, רכסים</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>32.74899</v>
+        <v>32.7551946</v>
       </c>
       <c r="C56" t="n">
-        <v>35.103904</v>
+        <v>35.1066628</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
@@ -1431,14 +1431,14 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>השקד 59, רכסים</t>
+          <t>הדקל 30, רכסים</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>32.7484557</v>
+        <v>32.7552473</v>
       </c>
       <c r="C57" t="n">
-        <v>35.1065067</v>
+        <v>35.1072159</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
@@ -1449,14 +1449,14 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>ורדים 5, רכסים</t>
+          <t>הורדים 4, רכסים</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>32.7558831</v>
+        <v>32.755216</v>
       </c>
       <c r="C58" t="n">
-        <v>35.0962669</v>
+        <v>35.0965091</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
@@ -1467,14 +1467,14 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>חזון איש 8, רכסים</t>
+          <t>הכלניות 1, רכסים</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>32.751478</v>
+        <v>32.7541406</v>
       </c>
       <c r="C59" t="n">
-        <v>35.104805</v>
+        <v>35.0975422</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
@@ -1485,14 +1485,14 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>כלניות 17, רכסים</t>
+          <t>הכלניות 32, רכסים</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>32.7537489</v>
+        <v>32.753939</v>
       </c>
       <c r="C60" t="n">
-        <v>35.0992594</v>
+        <v>35.09969299999999</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
@@ -1503,14 +1503,14 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>מעלה החזון איש 13, רכסים</t>
+          <t>הכלניות 47, רכסים</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>32.751018</v>
+        <v>32.7535253</v>
       </c>
       <c r="C61" t="n">
-        <v>35.104936</v>
+        <v>35.10205910000001</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
@@ -1521,14 +1521,14 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>רחוב הזית 13, רכסים</t>
+          <t>הנרקיסים 24, רכסים</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>32.7555378</v>
+        <v>32.7564592</v>
       </c>
       <c r="C62" t="n">
-        <v>35.101955</v>
+        <v>35.0993751</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
@@ -1539,14 +1539,14 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>רחוב סביון 38, רכסים</t>
+          <t>הרב קוק 12, רכסים</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>32.755329</v>
+        <v>32.7465011</v>
       </c>
       <c r="C63" t="n">
-        <v>35.1036374</v>
+        <v>35.1002575</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
@@ -1557,16 +1557,232 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
+          <t>הרב קוק 26, רכסים</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>32.7472521</v>
+      </c>
+      <c r="C64" t="n">
+        <v>35.1022188</v>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>הרימונים 16, רכסים</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>32.7499409</v>
+      </c>
+      <c r="C65" t="n">
+        <v>35.0985743</v>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>השקד 13, רכסים</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>32.752189</v>
+      </c>
+      <c r="C66" t="n">
+        <v>35.103784</v>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>השקד 14, רכסים</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>32.750799</v>
+      </c>
+      <c r="C67" t="n">
+        <v>35.102316</v>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>השקד 40, רכסים</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>32.74899</v>
+      </c>
+      <c r="C68" t="n">
+        <v>35.103904</v>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>השקד 59, רכסים</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>32.7484557</v>
+      </c>
+      <c r="C69" t="n">
+        <v>35.1065067</v>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>ורדים 5, רכסים</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>32.7558831</v>
+      </c>
+      <c r="C70" t="n">
+        <v>35.0962669</v>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>חזון איש 8, רכסים</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>32.751478</v>
+      </c>
+      <c r="C71" t="n">
+        <v>35.104805</v>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>כלניות 17, רכסים</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>32.7537489</v>
+      </c>
+      <c r="C72" t="n">
+        <v>35.0992594</v>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>מעלה החזון איש 13, רכסים</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>32.751018</v>
+      </c>
+      <c r="C73" t="n">
+        <v>35.104936</v>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>רחוב הזית 13, רכסים</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>32.7555378</v>
+      </c>
+      <c r="C74" t="n">
+        <v>35.101955</v>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>רחוב סביון 38, רכסים</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>32.755329</v>
+      </c>
+      <c r="C75" t="n">
+        <v>35.1036374</v>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
           <t>רימונים 15, רכסים</t>
         </is>
       </c>
-      <c r="B64" t="n">
+      <c r="B76" t="n">
         <v>32.7502502</v>
       </c>
-      <c r="C64" t="n">
+      <c r="C76" t="n">
         <v>35.0984128</v>
       </c>
-      <c r="D64" t="inlineStr">
+      <c r="D76" t="inlineStr">
         <is>
           <t>exact</t>
         </is>

</xml_diff>